<commit_message>
w4d: extract xlsx column widths and basic styles — wax-w4d5
</commit_message>
<xml_diff>
--- a/crates/wax-read/tests/fixtures/reader.xlsx
+++ b/crates/wax-read/tests/fixtures/reader.xlsx
@@ -30,11 +30,41 @@
     <numFmt numFmtId="164" formatCode="yyyy-mm-dd"/>
     <numFmt numFmtId="165" formatCode="0.0000 &quot;widgets&quot;"/>
   </numFmts>
-  <fonts count="1">
+  <fonts count="4">
     <font/>
+    <font>
+      <b/>
+      <i/>
+      <u/>
+      <strike/>
+      <sz val="13.5"/>
+      <name val="Aptos Display"/>
+      <color rgb="FF1A2B3C"/>
+    </font>
+    <font>
+      <color indexed="55"/>
+    </font>
+    <font>
+      <color theme="3" tint="-0.25"/>
+    </font>
   </fonts>
-  <fills count="1">
+  <fills count="4">
     <fill/>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFEEDDCC"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor indexed="24"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="4"/>
+      </patternFill>
+    </fill>
   </fills>
   <borders count="1">
     <border/>
@@ -44,10 +74,10 @@
   </cellStyleXfs>
   <cellXfs count="5">
     <xf numFmtId="0"/>
-    <xf numFmtId="14" applyNumberFormat="1"/>
-    <xf numFmtId="164" applyNumberFormat="1"/>
-    <xf numFmtId="4" applyNumberFormat="1"/>
-    <xf numFmtId="165" applyNumberFormat="1"/>
+    <xf numFmtId="14" fontId="1" fillId="1" applyNumberFormat="1"/>
+    <xf numFmtId="164" fontId="1" fillId="1" applyNumberFormat="1"/>
+    <xf numFmtId="4" fontId="2" fillId="2" applyNumberFormat="1"/>
+    <xf numFmtId="165" fontId="3" fillId="3" applyNumberFormat="1"/>
   </cellXfs>
 </styleSheet>
 </file>
@@ -55,6 +85,12 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <dimension ref="A1:G4"/>
+  <cols>
+    <col min="1" max="1" width="12.5" customWidth="1"/>
+    <col min="2" max="4" width="20" customWidth="true"/>
+    <col min="5" max="5" width="99" customWidth="false"/>
+    <col min="7" max="7" width="15.25" customWidth="1"/>
+  </cols>
   <sheetData>
     <row r="1">
       <c r="A1" t="s">

</xml_diff>